<commit_message>
fix: document Steamboat BPS place absence
</commit_message>
<xml_diff>
--- a/output/routt_absorption_workbook.xlsx
+++ b/output/routt_absorption_workbook.xlsx
@@ -800,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -826,6 +826,26 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>routt_county_appears</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>steamboat_text_appears</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>colorado_records_scanned</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>match_keys</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>source_url</t>
         </is>
       </c>
@@ -843,6 +863,24 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>269</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>county_code=107;fips_place_code=73825;place_name=steamboat springs</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>https://www2.census.gov/econ/bps/Place/West%20Region/we2020a.txt</t>
         </is>
       </c>
@@ -860,6 +898,24 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>268</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>county_code=107;fips_place_code=73825;place_name=steamboat springs</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>https://www2.census.gov/econ/bps/Place/West%20Region/we2021a.txt</t>
         </is>
       </c>
@@ -877,6 +933,24 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>268</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>county_code=107;fips_place_code=73825;place_name=steamboat springs</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>https://www2.census.gov/econ/bps/Place/West%20Region/we2022a.txt</t>
         </is>
       </c>
@@ -894,6 +968,24 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>268</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>county_code=107;fips_place_code=73825;place_name=steamboat springs</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>https://www2.census.gov/econ/bps/Place/West%20Region/we2023a.txt</t>
         </is>
       </c>
@@ -911,6 +1003,24 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>268</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>county_code=107;fips_place_code=73825;place_name=steamboat springs</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>https://www2.census.gov/econ/bps/Place/West%20Region/we2024a.txt</t>
         </is>
       </c>
@@ -927,6 +1037,24 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>270</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>county_code=107;fips_place_code=73825;place_name=steamboat springs</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>https://www2.census.gov/econ/bps/Place/West%20Region/we2025a.txt</t>
         </is>

</xml_diff>